<commit_message>
Use distinct series colors in the workbook charts
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fZhdaB5wDkT1uiYpGXgS4
</commit_message>
<xml_diff>
--- a/finance/Time_Value_of_Money_Models.xlsx
+++ b/finance/Time_Value_of_Money_Models.xlsx
@@ -2065,7 +2065,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFF9F9F9"/>
+        <bgColor rgb="FFEDE7F6"/>
       </patternFill>
     </fill>
     <fill>
@@ -2356,7 +2356,7 @@
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFD62728"/>
+      <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -2365,17 +2365,17 @@
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFB24543"/>
+      <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBFBF"/>
       <rgbColor rgb="FF878787"/>
       <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF953B38"/>
-      <rgbColor rgb="FFF9F9F9"/>
+      <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFF2F2F2"/>
+      <rgbColor rgb="FFEDE7F6"/>
       <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFD09493"/>
+      <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF1F77B4"/>
       <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
@@ -2387,27 +2387,27 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFEDE7F6"/>
+      <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFC6EFCE"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFD4A5A4"/>
+      <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFD9B0B0"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFBE4B48"/>
+      <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF595959"/>
-      <rgbColor rgb="FFC77978"/>
+      <rgbColor rgb="FF9467BD"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF2CA02C"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FFAB4744"/>
-      <rgbColor rgb="FF9D3E3B"/>
+      <rgbColor rgb="FFD62728"/>
+      <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF5B2C8F"/>
       <rgbColor rgb="FF333333"/>
     </indexedColors>
@@ -2475,11 +2475,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="953b38"/>
+              <a:srgbClr val="1f77b4"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="953b38"/>
+                <a:srgbClr val="1f77b4"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -2673,11 +2673,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="b24543"/>
+              <a:srgbClr val="d62728"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="b24543"/>
+                <a:srgbClr val="d62728"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -2871,11 +2871,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="c77978"/>
+              <a:srgbClr val="2ca02c"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="c77978"/>
+                <a:srgbClr val="2ca02c"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -3069,11 +3069,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="d9b0b0"/>
+              <a:srgbClr val="9467bd"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="d9b0b0"/>
+                <a:srgbClr val="9467bd"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -3259,11 +3259,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="26213681"/>
-        <c:axId val="13297976"/>
+        <c:axId val="57810076"/>
+        <c:axId val="31124134"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="26213681"/>
+        <c:axId val="57810076"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3329,7 +3329,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13297976"/>
+        <c:crossAx val="31124134"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3337,7 +3337,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="13297976"/>
+        <c:axId val="31124134"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3413,7 +3413,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26213681"/>
+        <c:crossAx val="57810076"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3525,11 +3525,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="953b38"/>
+              <a:srgbClr val="1f77b4"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="953b38"/>
+                <a:srgbClr val="1f77b4"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -3723,11 +3723,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="b24543"/>
+              <a:srgbClr val="d62728"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="b24543"/>
+                <a:srgbClr val="d62728"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -3921,11 +3921,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="c77978"/>
+              <a:srgbClr val="2ca02c"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="c77978"/>
+                <a:srgbClr val="2ca02c"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -4119,11 +4119,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="d9b0b0"/>
+              <a:srgbClr val="9467bd"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="d9b0b0"/>
+                <a:srgbClr val="9467bd"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -4309,11 +4309,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="90121420"/>
-        <c:axId val="65746206"/>
+        <c:axId val="46572462"/>
+        <c:axId val="19919812"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="90121420"/>
+        <c:axId val="46572462"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4379,7 +4379,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65746206"/>
+        <c:crossAx val="19919812"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4387,7 +4387,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="65746206"/>
+        <c:axId val="19919812"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4463,7 +4463,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90121420"/>
+        <c:crossAx val="46572462"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4576,13 +4576,12 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="ab4744"/>
+              <a:srgbClr val="1f77b4"/>
             </a:solidFill>
-            <a:ln w="9360">
+            <a:ln w="0">
               <a:solidFill>
-                <a:srgbClr val="f9f9f9"/>
+                <a:srgbClr val="1f77b4"/>
               </a:solidFill>
-              <a:round/>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
@@ -4690,13 +4689,12 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="d09493"/>
+              <a:srgbClr val="d62728"/>
             </a:solidFill>
-            <a:ln w="9360">
+            <a:ln w="0">
               <a:solidFill>
-                <a:srgbClr val="f9f9f9"/>
+                <a:srgbClr val="d62728"/>
               </a:solidFill>
-              <a:round/>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
@@ -4805,11 +4803,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="77056397"/>
-        <c:axId val="71633502"/>
+        <c:axId val="81112526"/>
+        <c:axId val="71148977"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="77056397"/>
+        <c:axId val="81112526"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4875,7 +4873,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71633502"/>
+        <c:crossAx val="71148977"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4883,7 +4881,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="71633502"/>
+        <c:axId val="71148977"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4959,7 +4957,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77056397"/>
+        <c:crossAx val="81112526"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5071,11 +5069,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="953b38"/>
+              <a:srgbClr val="1f77b4"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="953b38"/>
+                <a:srgbClr val="1f77b4"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -5743,11 +5741,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="b24543"/>
+              <a:srgbClr val="d62728"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="b24543"/>
+                <a:srgbClr val="d62728"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -6415,11 +6413,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="c77978"/>
+              <a:srgbClr val="2ca02c"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="c77978"/>
+                <a:srgbClr val="2ca02c"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -7087,11 +7085,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="d9b0b0"/>
+              <a:srgbClr val="9467bd"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="d9b0b0"/>
+                <a:srgbClr val="9467bd"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -7751,11 +7749,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="53786449"/>
-        <c:axId val="33294660"/>
+        <c:axId val="95290367"/>
+        <c:axId val="18200317"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="53786449"/>
+        <c:axId val="95290367"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7821,7 +7819,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33294660"/>
+        <c:crossAx val="18200317"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7829,7 +7827,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="33294660"/>
+        <c:axId val="18200317"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7905,7 +7903,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53786449"/>
+        <c:crossAx val="95290367"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8017,11 +8015,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="9d3e3b"/>
+              <a:srgbClr val="1f77b4"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="9d3e3b"/>
+                <a:srgbClr val="1f77b4"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -8809,11 +8807,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="be4b48"/>
+              <a:srgbClr val="d62728"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="be4b48"/>
+                <a:srgbClr val="d62728"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -9601,11 +9599,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="d4a5a4"/>
+              <a:srgbClr val="2ca02c"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="d4a5a4"/>
+                <a:srgbClr val="2ca02c"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -10385,11 +10383,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="17228911"/>
-        <c:axId val="47733216"/>
+        <c:axId val="52009787"/>
+        <c:axId val="78651433"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="17228911"/>
+        <c:axId val="52009787"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10455,7 +10453,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47733216"/>
+        <c:crossAx val="78651433"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -10463,7 +10461,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="47733216"/>
+        <c:axId val="78651433"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10539,7 +10537,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17228911"/>
+        <c:crossAx val="52009787"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -10651,11 +10649,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="953b38"/>
+              <a:srgbClr val="1f77b4"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="953b38"/>
+                <a:srgbClr val="1f77b4"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -10849,11 +10847,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="b24543"/>
+              <a:srgbClr val="d62728"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="b24543"/>
+                <a:srgbClr val="d62728"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -11047,11 +11045,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="c77978"/>
+              <a:srgbClr val="2ca02c"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="c77978"/>
+                <a:srgbClr val="2ca02c"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -11245,11 +11243,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="d9b0b0"/>
+              <a:srgbClr val="9467bd"/>
             </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="25560">
               <a:solidFill>
-                <a:srgbClr val="d9b0b0"/>
+                <a:srgbClr val="9467bd"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -11435,11 +11433,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="46482767"/>
-        <c:axId val="22575704"/>
+        <c:axId val="15240186"/>
+        <c:axId val="4014952"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="46482767"/>
+        <c:axId val="15240186"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11505,7 +11503,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22575704"/>
+        <c:crossAx val="4014952"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -11513,7 +11511,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="22575704"/>
+        <c:axId val="4014952"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11589,7 +11587,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46482767"/>
+        <c:crossAx val="15240186"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>